<commit_message>
Aplica o design system Saiaê v1.0 nas duas planilhas
Mostarda #FFC21A como destaque (texto sempre tinta), tinta #18171C,
papel #F6F5F2, Outfit + Figtree e cores de status do sistema.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011pEscwW9GNGpmNb8Mg2awf
</commit_message>
<xml_diff>
--- a/Mesa_Agil_Enxuta.xlsx
+++ b/Mesa_Agil_Enxuta.xlsx
@@ -115,7 +115,7 @@
     <t xml:space="preserve">PREMISSAS  ·  PREENCHA UMA VEZ</t>
   </si>
   <si>
-    <t xml:space="preserve">Campos VERDE-CLAROS = você preenche. Preços vieram do escopo; o resto são exemplos para trocar pelos seus números.</t>
+    <t xml:space="preserve">Campos AMARELO-CLAROS = você preenche. Preços vieram do escopo; o resto são exemplos para trocar pelos seus números.</t>
   </si>
   <si>
     <t xml:space="preserve">GERAL</t>
@@ -289,7 +289,7 @@
     <t xml:space="preserve">MEU MÊS  ·  O QUE ACONTECEU DE VERDADE</t>
   </si>
   <si>
-    <t xml:space="preserve">No fim de cada mês, preencha os 6 campos verde-claros da linha do mês. O resto compara com a projeção sozinho.</t>
+    <t xml:space="preserve">No fim de cada mês, preencha os 6 campos amarelo-claros da linha do mês. O resto compara com a projeção sozinho.</t>
   </si>
   <si>
     <t xml:space="preserve">VOCÊ LANÇA</t>
@@ -385,7 +385,7 @@
     <numFmt numFmtId="183" formatCode="#,##0.0;\-#,##0.0;\-"/>
     <numFmt numFmtId="184" formatCode="0"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,78 +411,70 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF0F172A"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF18171C"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Space Grotesk"/>
+      <name val="Outfit"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF64748B"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF5E5C66"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Space Grotesk"/>
+      <sz val="11"/>
+      <color rgb="FF18171C"/>
+      <name val="Outfit"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FF006948"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF5E5C66"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF64748B"/>
-      <name val="Space Grotesk"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="20"/>
-      <color rgb="FF0F172A"/>
-      <name val="Space Grotesk"/>
+      <sz val="22"/>
+      <color rgb="FF18171C"/>
+      <name val="Outfit"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF0F172A"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF18171C"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
-      <color rgb="FF64748B"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF5E5C66"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF0F172A"/>
-      <name val="Space Grotesk"/>
+      <sz val="12"/>
+      <color rgb="FF18171C"/>
+      <name val="Outfit"/>
       <family val="2"/>
     </font>
     <font>
@@ -493,32 +485,24 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Space Grotesk"/>
+      <name val="Outfit"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF0F172A"/>
-      <name val="Space Grotesk"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF065F46"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF18171C"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FF0F172A"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF18171C"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -526,30 +510,30 @@
       <b val="true"/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Space Grotesk"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF64748B"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF5E5C66"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FFD97706"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FFA34E00"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="8"/>
-      <color rgb="FF64748B"/>
-      <name val="Space Grotesk"/>
+      <color rgb="FF5E5C66"/>
+      <name val="Figtree"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -563,48 +547,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFF6F5F2"/>
+        <bgColor rgb="FFFFF8E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF6F5F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF006948"/>
-        <bgColor rgb="FF065F46"/>
+        <fgColor rgb="FF18171C"/>
+        <bgColor rgb="FF2E2C35"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD97706"/>
-        <bgColor rgb="FFFF9900"/>
+        <fgColor rgb="FFFFC21A"/>
+        <bgColor rgb="FFE6A800"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFECFDF5"/>
-        <bgColor rgb="FFF1F5F9"/>
+        <fgColor rgb="FFFFF8E1"/>
+        <bgColor rgb="FFF6F5F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-        <bgColor rgb="FFF8FAFC"/>
+        <fgColor rgb="FFECEAE6"/>
+        <bgColor rgb="FFFDE7E4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00855D"/>
-        <bgColor rgb="FF059669"/>
+        <fgColor rgb="FF2E2C35"/>
+        <bgColor rgb="FF333300"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -614,49 +598,58 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </left>
       <right/>
       <top style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FFFFC21A"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFD97706"/>
+        <color rgb="FFFFC21A"/>
       </left>
       <right/>
       <top style="thin">
-        <color rgb="FFD97706"/>
+        <color rgb="FFFFC21A"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD97706"/>
+        <color rgb="FFFFC21A"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </right>
       <top style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </right>
       <top/>
       <bottom/>
@@ -664,74 +657,74 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </left>
       <right style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </right>
       <top style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FF10B981"/>
+        <color rgb="FFE6A800"/>
       </left>
       <right style="thin">
-        <color rgb="FF10B981"/>
+        <color rgb="FFE6A800"/>
       </right>
       <top style="thin">
-        <color rgb="FF10B981"/>
+        <color rgb="FFE6A800"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF10B981"/>
+        <color rgb="FFE6A800"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </right>
       <top style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </right>
       <top style="medium">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFB5B3BB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE2E8F0"/>
+        <color rgb="FFD9D7DC"/>
       </bottom>
       <diagonal/>
     </border>
@@ -774,223 +767,223 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="178" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="178" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="179" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="182" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="182" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="183" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="183" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="182" fontId="10" fillId="7" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="182" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="184" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="182" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="183" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="183" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="184" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="183" fontId="10" fillId="7" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="182" fontId="16" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="183" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="183" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="182" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="182" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="184" fontId="16" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="16" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="183" fontId="16" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="183" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="184" fontId="20" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="183" fontId="11" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1006,32 +999,32 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FFEF4444"/>
+        <color rgb="FFB22514"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF059669"/>
+        <color rgb="FF0E7A40"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="FF991B1B"/>
+        <color rgb="FFB22514"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFEF2F2"/>
+          <bgColor rgb="FFFDE7E4"/>
         </patternFill>
       </fill>
       <border diagonalUp="false" diagonalDown="false">
         <left/>
         <right/>
         <top style="thin">
-          <color rgb="FFFCA5A5"/>
+          <color rgb="FFF0412F"/>
         </top>
         <bottom style="thin">
-          <color rgb="FFFCA5A5"/>
+          <color rgb="FFF0412F"/>
         </bottom>
         <diagonal/>
       </border>
@@ -1039,21 +1032,21 @@
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="FF065F46"/>
+        <color rgb="FF0E7A40"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFECFDF5"/>
+          <bgColor rgb="FFE3F7EC"/>
         </patternFill>
       </fill>
       <border diagonalUp="false" diagonalDown="false">
         <left/>
         <right/>
         <top style="thin">
-          <color rgb="FF10B981"/>
+          <color rgb="FF1FBF6A"/>
         </top>
         <bottom style="thin">
-          <color rgb="FF10B981"/>
+          <color rgb="FF1FBF6A"/>
         </bottom>
         <diagonal/>
       </border>
@@ -1070,53 +1063,53 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF006948"/>
+      <rgbColor rgb="FF0E7A40"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF00855D"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFB5B3BB"/>
       <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FFEF4444"/>
-      <rgbColor rgb="FFFEF2F2"/>
-      <rgbColor rgb="FFECFDF5"/>
+      <rgbColor rgb="FFA34E00"/>
+      <rgbColor rgb="FFFFF8E1"/>
+      <rgbColor rgb="FFE3F7EC"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCBD5E1"/>
+      <rgbColor rgb="FFD9D7DC"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF059669"/>
+      <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFF1F5F9"/>
-      <rgbColor rgb="FFE2E8F0"/>
-      <rgbColor rgb="FFF8FAFC"/>
+      <rgbColor rgb="FFF6F5F2"/>
+      <rgbColor rgb="FFECEAE6"/>
+      <rgbColor rgb="FFFDE7E4"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFCA5A5"/>
+      <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFD97706"/>
-      <rgbColor rgb="FF64748B"/>
-      <rgbColor rgb="FF94A3B8"/>
-      <rgbColor rgb="FF065F46"/>
-      <rgbColor rgb="FF10B981"/>
-      <rgbColor rgb="FF0F172A"/>
+      <rgbColor rgb="FFFFC21A"/>
+      <rgbColor rgb="FFE6A800"/>
+      <rgbColor rgb="FFF0412F"/>
+      <rgbColor rgb="FF5E5C66"/>
+      <rgbColor rgb="FF8A8893"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF1FBF6A"/>
+      <rgbColor rgb="FF18171C"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF991B1B"/>
+      <rgbColor rgb="FFB22514"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF2E2C35"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1134,19 +1127,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="1" sz="1100" spc="-1" strike="noStrike">
+              <a:defRPr b="1" sz="1200" spc="-1" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="0f172a"/>
+                  <a:srgbClr val="18171c"/>
                 </a:solidFill>
-                <a:latin typeface="Space Grotesk"/>
+                <a:latin typeface="Outfit"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="1" sz="1100" spc="-1" strike="noStrike">
+              <a:rPr b="1" sz="1200" spc="-1" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="0f172a"/>
+                  <a:srgbClr val="18171c"/>
                 </a:solidFill>
-                <a:latin typeface="Space Grotesk"/>
+                <a:latin typeface="Outfit"/>
               </a:rPr>
               <a:t>Clientes ativos: plano × real</a:t>
             </a:r>
@@ -1182,11 +1175,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="94a3b8"/>
+              <a:srgbClr val="8a8893"/>
             </a:solidFill>
             <a:ln w="28080">
               <a:solidFill>
-                <a:srgbClr val="94a3b8"/>
+                <a:srgbClr val="8a8893"/>
               </a:solidFill>
               <a:prstDash val="dash"/>
               <a:round/>
@@ -1399,11 +1392,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="059669"/>
+              <a:srgbClr val="e6a800"/>
             </a:solidFill>
             <a:ln w="32040">
               <a:solidFill>
-                <a:srgbClr val="059669"/>
+                <a:srgbClr val="e6a800"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1413,7 +1406,7 @@
             <c:size val="6"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="059669"/>
+                <a:srgbClr val="e6a800"/>
               </a:solidFill>
             </c:spPr>
           </c:marker>
@@ -1544,11 +1537,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="41527187"/>
-        <c:axId val="27073084"/>
+        <c:axId val="19249189"/>
+        <c:axId val="75253835"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="41527187"/>
+        <c:axId val="19249189"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1580,7 +1573,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27073084"/>
+        <c:crossAx val="75253835"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1588,7 +1581,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27073084"/>
+        <c:axId val="75253835"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1598,7 +1591,7 @@
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="e2e8f0"/>
+                <a:srgbClr val="d9d7dc"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1630,7 +1623,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41527187"/>
+        <c:crossAx val="19249189"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1674,7 +1667,7 @@
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="e2e8f0"/>
+        <a:srgbClr val="d9d7dc"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -1694,19 +1687,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="1" sz="1100" spc="-1" strike="noStrike">
+              <a:defRPr b="1" sz="1200" spc="-1" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="0f172a"/>
+                  <a:srgbClr val="18171c"/>
                 </a:solidFill>
-                <a:latin typeface="Space Grotesk"/>
+                <a:latin typeface="Outfit"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="1" sz="1100" spc="-1" strike="noStrike">
+              <a:rPr b="1" sz="1200" spc="-1" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="0f172a"/>
+                  <a:srgbClr val="18171c"/>
                 </a:solidFill>
-                <a:latin typeface="Space Grotesk"/>
+                <a:latin typeface="Outfit"/>
               </a:rPr>
               <a:t>Caixa acumulado (plano)</a:t>
             </a:r>
@@ -1742,11 +1735,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="059669"/>
+              <a:srgbClr val="e6a800"/>
             </a:solidFill>
             <a:ln w="28080">
               <a:solidFill>
-                <a:srgbClr val="059669"/>
+                <a:srgbClr val="e6a800"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1950,11 +1943,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="39068488"/>
-        <c:axId val="63417775"/>
+        <c:axId val="55710498"/>
+        <c:axId val="85747787"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="39068488"/>
+        <c:axId val="55710498"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1986,7 +1979,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63417775"/>
+        <c:crossAx val="85747787"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1994,7 +1987,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63417775"/>
+        <c:axId val="85747787"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2004,7 +1997,7 @@
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="e2e8f0"/>
+                <a:srgbClr val="d9d7dc"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2036,7 +2029,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39068488"/>
+        <c:crossAx val="55710498"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2056,7 +2049,7 @@
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="e2e8f0"/>
+        <a:srgbClr val="d9d7dc"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -2077,7 +2070,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>959040</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2085,7 +2078,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="266760" y="3962520"/>
+        <a:off x="266760" y="4019400"/>
         <a:ext cx="5759640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2107,7 +2100,7 @@
       <xdr:col>16</xdr:col>
       <xdr:colOff>959040</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2115,7 +2108,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7467480" y="3962520"/>
+        <a:off x="7467480" y="4019400"/>
         <a:ext cx="5759640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2307,7 +2300,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF006948"/>
+    <tabColor rgb="FF18171C"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AA63"/>
@@ -2363,7 +2356,7 @@
       <c r="Z1" s="1"/>
       <c r="AA1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="str">
         <f aca="false">"MESA ÁGIL  ·  PAINEL  ·  CENÁRIO "&amp;UPPER(Premissas!$C$8)</f>
@@ -4411,7 +4404,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFD97706"/>
+    <tabColor rgb="FFFFC21A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:M68"/>
@@ -4440,7 +4433,7 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="26" t="s">
         <v>29</v>
@@ -5727,7 +5720,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF64748B"/>
+    <tabColor rgb="FF5E5C66"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:T57"/>
@@ -5763,7 +5756,7 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="26" t="s">
         <v>87</v>
@@ -7613,7 +7606,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF64748B"/>
+    <tabColor rgb="FF5E5C66"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R55"/>
@@ -7648,7 +7641,7 @@
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="26" t="str">
         <f aca="false">"PROJEÇÃO 24 MESES  ·  CENÁRIO "&amp;UPPER(Premissas!$C$8)</f>

</xml_diff>